<commit_message>
POM with @FindBy, @FindBys, @FindAll and dynamic xpath
</commit_message>
<xml_diff>
--- a/vtiger-crm-automation-framework-m10/src/test/resources/testScriptData.xlsx
+++ b/vtiger-crm-automation-framework-m10/src/test/resources/testScriptData.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="150">
   <si>
     <t>Organization Name</t>
   </si>
@@ -465,6 +465,12 @@
   </si>
   <si>
     <t>upadhyay</t>
+  </si>
+  <si>
+    <t>vtiger429</t>
+  </si>
+  <si>
+    <t>Vtiger813</t>
   </si>
 </sst>
 </file>
@@ -818,7 +824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -1354,6 +1360,44 @@
         <v>41</v>
       </c>
     </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>